<commit_message>
test(auth): implement TC05 - verify error message for username with special characters
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -606,6 +606,33 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>@@@###</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Username chứa ký tự đặc biệt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC03 - verify validation message for empty username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -556,6 +556,29 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Username rỗng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC01 - verify successful login with valid credentials
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,33 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TC01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_USERNAME&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Đăng nhập với tài khoản hợp lệ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC04 - verify validation error for whitespace-only username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Username chỉ có khoảng trắng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC02 - verify error message for non-existent username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,33 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>username_not_exist</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Username không tồn tại</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC06 - verify error message for incorrect password
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -633,6 +633,33 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>huongnt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>wrong_password</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Password sai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC08 - verify validation error for whitespace-only password
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,33 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>huongnt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Password chỉ có khoảng trắng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC09 - verify validation message when both username and password are empty
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -710,6 +710,25 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Username và Password đều rỗng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(security): implement TC11 - verify injection protection against SQL injection in username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -756,6 +756,33 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>' OR '1'='1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SQL Injection trong Username</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC10 - verify error message when both username and password are invalid
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -729,6 +729,33 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>username_not_exist</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>wrong_password</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cả Username và Password đều sai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(auth): implement TC07 - verify validation message for empty password
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,29 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>huongnt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Password rỗng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(boundary): implement TC16 - verify boundary validation for maximum length password (256 characters)
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -891,6 +891,33 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_USERNAME&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Password quá dài (256 ký tự)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(security): implement TC13 - verify security protection against XSS attack in username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -810,6 +810,33 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>XSS attack trong Username</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(format): implement TC17 - verify validation for email address format username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,33 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>test@gmail.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Username dạng email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(boundary): implement TC14 - verify boundary validation for single character username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -837,6 +837,33 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Username 1 ký tự (quá ngắn)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(security): implement TC12 - verify injection protection against SQL injection in password
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -783,6 +783,33 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_USERNAME&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>' OR '1'='1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SQL Injection trong Password</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(boundary): implement TC15 - verify boundary validation for maximum length username (256 characters)
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -864,6 +864,33 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Username quá dài (256 ký tự)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(format): implement TC19 - verify validation for numeric-only username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -972,6 +972,33 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Username toàn số</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(format): implement TC20 - verify rejection of password containing space character
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -999,6 +999,33 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>huongnt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>pass word 123</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Password có khoảng trắng ở giữa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test(format): implement TC18 - verify validation for unaccented Vietnamese username
</commit_message>
<xml_diff>
--- a/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
+++ b/UTC-Selenium-Test/src/test/resources/LoginTestData.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -945,6 +945,33 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nguyenvanan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>&lt;&lt;VALID_PASSWORD&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Username tiếng Việt không dấu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>